<commit_message>
Update DateBase/orders/Dang Nguyen 195_2026-10-13.xlsx
</commit_message>
<xml_diff>
--- a/DateBase/orders/Dang Nguyen 195_2026-10-13.xlsx
+++ b/DateBase/orders/Dang Nguyen 195_2026-10-13.xlsx
@@ -524,7 +524,10 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>5</v>
+        <v>53</v>
+      </c>
+      <c r="C11" t="str">
+        <v>144_高原红_High Plateau Red_Rosa rugosa Thunb._20stems</v>
       </c>
     </row>
   </sheetData>

</xml_diff>